<commit_message>
feat: Hoan thien he thong phan quyen Truong Khoa/Bo Mon, sua loi 404 doi mat khau va dong bo toan dien du lieu
</commit_message>
<xml_diff>
--- a/sample_imports/01_Khoa_Mau.xlsx
+++ b/sample_imports/01_Khoa_Mau.xlsx
@@ -7,7 +7,7 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="DuLieuMau" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -15,10 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
-  <si>
-    <t>MẪU DỮ LIỆU KHOA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="84">
   <si>
     <t>MaKhoa</t>
   </si>
@@ -32,28 +29,244 @@
     <t>MoTa</t>
   </si>
   <si>
+    <t>CNTT</t>
+  </si>
+  <si>
+    <t>Khoa Công nghệ Thông tin</t>
+  </si>
+  <si>
+    <t>PGS.TS. Nguyễn Văn Hùng</t>
+  </si>
+  <si>
+    <t>Khoa đào tạo CNTT, CNPM, HTTT, KHMT, ATTT, MMT</t>
+  </si>
+  <si>
+    <t>QTKD</t>
+  </si>
+  <si>
+    <t>Khoa Quản trị Kinh doanh</t>
+  </si>
+  <si>
+    <t>PGS.TS. Trần Đình Nam</t>
+  </si>
+  <si>
+    <t>Khoa Quản trị kinh doanh và Marketing</t>
+  </si>
+  <si>
+    <t>TP</t>
+  </si>
+  <si>
+    <t>Khoa Công nghệ Thực phẩm</t>
+  </si>
+  <si>
+    <t>GS.TS. Lê Thị Mai</t>
+  </si>
+  <si>
+    <t>Khoa Công nghệ thực phẩm và Dinh dưỡng</t>
+  </si>
+  <si>
+    <t>DDT</t>
+  </si>
+  <si>
+    <t>Khoa Điện - Điện tử</t>
+  </si>
+  <si>
+    <t>PGS.TS. Vũ Trọng Hưng</t>
+  </si>
+  <si>
+    <t>Khoa Kỹ thuật Điện, Điện tử viễn thông, Tự động hóa</t>
+  </si>
+  <si>
+    <t>CK</t>
+  </si>
+  <si>
+    <t>Khoa Cơ khí - Chế tạo máy</t>
+  </si>
+  <si>
+    <t>PGS.TS. Đặng Quốc Thịnh</t>
+  </si>
+  <si>
+    <t>Khoa Cơ khí động lực, Cơ điện tử, Chế tạo máy</t>
+  </si>
+  <si>
     <t>NN</t>
   </si>
   <si>
-    <t>Khoa Ngoại Ngữ</t>
-  </si>
-  <si>
-    <t>TS. Lê Thị Mai</t>
-  </si>
-  <si>
-    <t>Khoa Ngoại ngữ trường Đại học Công Thương</t>
-  </si>
-  <si>
-    <t>QTKD</t>
-  </si>
-  <si>
-    <t>Khoa Quản Trị Kinh Doanh</t>
-  </si>
-  <si>
-    <t>PGS.TS Hoàng Đình Tuấn</t>
-  </si>
-  <si>
-    <t>Khoa Quản trị kinh doanh trường Đại học Công Thương</t>
+    <t>Khoa Ngoại ngữ</t>
+  </si>
+  <si>
+    <t>TS. Phạm Thị Bích Loan</t>
+  </si>
+  <si>
+    <t>Khoa Ngôn ngữ Anh, Tiếng Trung, Tiếng Nhật</t>
+  </si>
+  <si>
+    <t>KTTC</t>
+  </si>
+  <si>
+    <t>Khoa Kế toán - Tài chính</t>
+  </si>
+  <si>
+    <t>PGS.TS. Ngô Xuân Hiếu</t>
+  </si>
+  <si>
+    <t>Khoa Kế toán doanh nghiệp, Kiểm toán và Tài chính</t>
+  </si>
+  <si>
+    <t>LUAT</t>
+  </si>
+  <si>
+    <t>Khoa Luật</t>
+  </si>
+  <si>
+    <t>TS. Phan Văn Phúc</t>
+  </si>
+  <si>
+    <t>Khoa Luật kinh tế và Luật thương mại quốc tế</t>
+  </si>
+  <si>
+    <t>SH</t>
+  </si>
+  <si>
+    <t>Khoa Công nghệ Sinh học</t>
+  </si>
+  <si>
+    <t>PGS.TS. Đỗ Hoài Nam</t>
+  </si>
+  <si>
+    <t>Khoa Sinh học ứng dụng và Kỹ thuật y sinh</t>
+  </si>
+  <si>
+    <t>HH</t>
+  </si>
+  <si>
+    <t>Khoa Hóa học &amp; Công nghệ Hóa</t>
+  </si>
+  <si>
+    <t>TS. Dương Văn Cường</t>
+  </si>
+  <si>
+    <t>Khoa Công nghệ kỹ thuật Hóa học và Vật liệu polyme</t>
+  </si>
+  <si>
+    <t>DL</t>
+  </si>
+  <si>
+    <t>Khoa Du lịch &amp; Khách sạn</t>
+  </si>
+  <si>
+    <t>TS. Hoàng Yến Linh</t>
+  </si>
+  <si>
+    <t>Khoa Quản trị dịch vụ du lịch, Lữ hành và Khách sạn</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>Khoa Môi trường &amp; Tài nguyên</t>
+  </si>
+  <si>
+    <t>TS. Bùi Mai Hoa</t>
+  </si>
+  <si>
+    <t>Khoa Khoa học Môi trường và Quản lý tài nguyên</t>
+  </si>
+  <si>
+    <t>TOAN</t>
+  </si>
+  <si>
+    <t>Khoa Toán - Thống kê</t>
+  </si>
+  <si>
+    <t>TS. Lê Hải Đăng</t>
+  </si>
+  <si>
+    <t>Khoa Toán ứng dụng, Khoa học dữ liệu</t>
+  </si>
+  <si>
+    <t>KTS</t>
+  </si>
+  <si>
+    <t>Khoa Kiến trúc - Mỹ thuật</t>
+  </si>
+  <si>
+    <t>TS. Phạm Minh Tuấn</t>
+  </si>
+  <si>
+    <t>Khoa Kiến trúc công trình và Thiết kế đồ họa</t>
+  </si>
+  <si>
+    <t>XD</t>
+  </si>
+  <si>
+    <t>Khoa Kỹ thuật Xây dựng</t>
+  </si>
+  <si>
+    <t>TS. Nguyễn Hoàng Long</t>
+  </si>
+  <si>
+    <t>Khoa Xây dựng dân dụng và Công trình giao thông</t>
+  </si>
+  <si>
+    <t>TMDT</t>
+  </si>
+  <si>
+    <t>Khoa Thương mại Điện tử</t>
+  </si>
+  <si>
+    <t>TS. Võ Duy Hùng</t>
+  </si>
+  <si>
+    <t>Khoa Kinh tế số và Thương mại điện tử</t>
+  </si>
+  <si>
+    <t>TC</t>
+  </si>
+  <si>
+    <t>Khoa Tài chính - Ngân hàng</t>
+  </si>
+  <si>
+    <t>PGS.TS. Nguyễn Hồng Phong</t>
+  </si>
+  <si>
+    <t>Khoa Thị trường vốn, Chứng khoán và Fintech</t>
+  </si>
+  <si>
+    <t>TT</t>
+  </si>
+  <si>
+    <t>Khoa Truyền thông &amp; Quan hệ công chúng</t>
+  </si>
+  <si>
+    <t>TS. Lương Thu Thảo</t>
+  </si>
+  <si>
+    <t>Khoa Quan hệ công chúng và Báo chí truyền thông</t>
+  </si>
+  <si>
+    <t>LOG</t>
+  </si>
+  <si>
+    <t>Khoa Logistics &amp; Chuỗi cung ứng</t>
+  </si>
+  <si>
+    <t>PGS.TS. Mai Thế Vinh</t>
+  </si>
+  <si>
+    <t>Khoa Logistics và Quản trị chuỗi cung ứng toàn cầu</t>
+  </si>
+  <si>
+    <t>ATTT</t>
+  </si>
+  <si>
+    <t>Khoa An toàn Thông tin &amp; Mạng</t>
+  </si>
+  <si>
+    <t>TS. Trịnh Văn Thành</t>
+  </si>
+  <si>
+    <t>Khoa An toàn an ninh mạng và Mật mã học</t>
   </si>
 </sst>
 </file>
@@ -61,7 +274,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -71,52 +284,16 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="13"/>
-      <color rgb="FF1E3A8A"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1E40AF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -124,54 +301,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF93C5FD"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF93C5FD"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF93C5FD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF93C5FD"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFE2E8F0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFE2E8F0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE2E8F0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFE2E8F0"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="1">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="3" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="2" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,66 +606,310 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="10.426" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="45.846" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="30.564" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="61.271" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" customHeight="1" ht="28">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" customHeight="1" ht="24">
-      <c r="A2" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" customHeight="1" ht="20">
-      <c r="A3" s="3" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" customHeight="1" ht="20">
-      <c r="A4" s="4" t="s">
+      <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
         <v>12</v>
       </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" t="s">
+        <v>82</v>
+      </c>
+      <c r="D21" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells>
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>

</xml_diff>